<commit_message>
Optimize .gitignore and prepare for push
</commit_message>
<xml_diff>
--- a/bin/数据采集配置.xlsx
+++ b/bin/数据采集配置.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\go-energy\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\go-energy\bin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E297F7-BAFB-4878-9004-B6B24C82102A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2669BBF-DED8-4F2D-B648-928AA37B5C9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="设备表" sheetId="19" r:id="rId1"/>
     <sheet name="配置表" sheetId="15" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">设备表!$A$1:$L$130</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">设备表!$A$1:$L$132</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="945" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="959" uniqueCount="207">
   <si>
     <t>编号</t>
   </si>
@@ -474,175 +474,200 @@
     <t>九号配电室</t>
   </si>
   <si>
+    <t>192.168.40.19</t>
+  </si>
+  <si>
+    <t>2号挤出机</t>
+  </si>
+  <si>
+    <t>4号挤出机</t>
+  </si>
+  <si>
+    <t>5号挤出机</t>
+  </si>
+  <si>
+    <t>6号挤出机</t>
+  </si>
+  <si>
+    <t>7号挤出机</t>
+  </si>
+  <si>
+    <t>8号挤出机</t>
+  </si>
+  <si>
+    <t>11号挤出机</t>
+  </si>
+  <si>
+    <t>14号冷却塔</t>
+  </si>
+  <si>
+    <t>192.168.59.21</t>
+  </si>
+  <si>
+    <t>15号冷却塔</t>
+  </si>
+  <si>
+    <t>192.168.59.22</t>
+  </si>
+  <si>
+    <t>7号环保设备</t>
+  </si>
+  <si>
+    <t>192.168.36.15</t>
+  </si>
+  <si>
+    <t>铜米机</t>
+  </si>
+  <si>
+    <t>1号悬臂单绞机</t>
+  </si>
+  <si>
+    <t>2号悬臂单绞机</t>
+  </si>
+  <si>
+    <t>桑普1000+1250电源1</t>
+  </si>
+  <si>
+    <t>桑普1000+1250电源2</t>
+  </si>
+  <si>
+    <t>3号成缆机</t>
+  </si>
+  <si>
+    <t>桑普1000绞线机</t>
+  </si>
+  <si>
+    <t>63号笼绞机</t>
+  </si>
+  <si>
+    <t>64号笼绞机</t>
+  </si>
+  <si>
+    <t>16号冷却塔</t>
+  </si>
+  <si>
+    <t>192.168.59.23</t>
+  </si>
+  <si>
+    <t>电子加速器</t>
+  </si>
+  <si>
+    <t>复绕机（电气值班室外）</t>
+  </si>
+  <si>
+    <t>三车间南侧照明（及办公室）</t>
+  </si>
+  <si>
+    <t>三车间北侧照明及行车电源</t>
+  </si>
+  <si>
+    <t>动力站</t>
+  </si>
+  <si>
+    <t>18号冷却塔</t>
+  </si>
+  <si>
+    <t>192.168.59.24</t>
+  </si>
+  <si>
+    <t>研发楼</t>
+  </si>
+  <si>
+    <t>1号变压器</t>
+  </si>
+  <si>
+    <t>2号变压器</t>
+  </si>
+  <si>
+    <t>3号变压器</t>
+  </si>
+  <si>
+    <t>4号变压器</t>
+  </si>
+  <si>
+    <t>5号变压器</t>
+  </si>
+  <si>
+    <t>6号变压器</t>
+  </si>
+  <si>
+    <t>7号变压器</t>
+  </si>
+  <si>
+    <t>8号变压器</t>
+  </si>
+  <si>
+    <t>9号变压器</t>
+  </si>
+  <si>
+    <t>十号配电室</t>
+  </si>
+  <si>
+    <t>10号变压器</t>
+  </si>
+  <si>
+    <t>USER</t>
+  </si>
+  <si>
+    <t>jldgxcx</t>
+  </si>
+  <si>
+    <t>PASSWORD</t>
+  </si>
+  <si>
+    <t>Jldg123654.</t>
+  </si>
+  <si>
+    <t>HOST</t>
+  </si>
+  <si>
+    <t>xs.jldg.com</t>
+  </si>
+  <si>
+    <t>DATABASE</t>
+  </si>
+  <si>
+    <t>192.168.40.19</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>二车间</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>七号配电室</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>二车间冷感机</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>二车间空压机</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>192.168.40.17</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>e20250529</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>9号挤出机</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>10号挤出机</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
     <t>1号挤出机</t>
-  </si>
-  <si>
-    <t>192.168.40.19</t>
-  </si>
-  <si>
-    <t>2号挤出机</t>
+    <phoneticPr fontId="8" type="noConversion"/>
   </si>
   <si>
     <t>3号挤出机</t>
-  </si>
-  <si>
-    <t>4号挤出机</t>
-  </si>
-  <si>
-    <t>5号挤出机</t>
-  </si>
-  <si>
-    <t>6号挤出机</t>
-  </si>
-  <si>
-    <t>7号挤出机</t>
-  </si>
-  <si>
-    <t>8号挤出机</t>
-  </si>
-  <si>
-    <t>9号挤出机</t>
-  </si>
-  <si>
-    <t>10号挤出机</t>
-  </si>
-  <si>
-    <t>11号挤出机</t>
-  </si>
-  <si>
-    <t>14号冷却塔</t>
-  </si>
-  <si>
-    <t>192.168.59.21</t>
-  </si>
-  <si>
-    <t>15号冷却塔</t>
-  </si>
-  <si>
-    <t>192.168.59.22</t>
-  </si>
-  <si>
-    <t>7号环保设备</t>
-  </si>
-  <si>
-    <t>192.168.36.15</t>
-  </si>
-  <si>
-    <t>铜米机</t>
-  </si>
-  <si>
-    <t>1号悬臂单绞机</t>
-  </si>
-  <si>
-    <t>2号悬臂单绞机</t>
-  </si>
-  <si>
-    <t>桑普1000+1250电源1</t>
-  </si>
-  <si>
-    <t>桑普1000+1250电源2</t>
-  </si>
-  <si>
-    <t>3号成缆机</t>
-  </si>
-  <si>
-    <t>桑普1000绞线机</t>
-  </si>
-  <si>
-    <t>63号笼绞机</t>
-  </si>
-  <si>
-    <t>64号笼绞机</t>
-  </si>
-  <si>
-    <t>16号冷却塔</t>
-  </si>
-  <si>
-    <t>192.168.59.23</t>
-  </si>
-  <si>
-    <t>电子加速器</t>
-  </si>
-  <si>
-    <t>复绕机（电气值班室外）</t>
-  </si>
-  <si>
-    <t>三车间南侧照明（及办公室）</t>
-  </si>
-  <si>
-    <t>三车间北侧照明及行车电源</t>
-  </si>
-  <si>
-    <t>动力站</t>
-  </si>
-  <si>
-    <t>18号冷却塔</t>
-  </si>
-  <si>
-    <t>192.168.59.24</t>
-  </si>
-  <si>
-    <t>研发楼</t>
-  </si>
-  <si>
-    <t>1号变压器</t>
-  </si>
-  <si>
-    <t>2号变压器</t>
-  </si>
-  <si>
-    <t>3号变压器</t>
-  </si>
-  <si>
-    <t>4号变压器</t>
-  </si>
-  <si>
-    <t>5号变压器</t>
-  </si>
-  <si>
-    <t>6号变压器</t>
-  </si>
-  <si>
-    <t>7号变压器</t>
-  </si>
-  <si>
-    <t>8号变压器</t>
-  </si>
-  <si>
-    <t>9号变压器</t>
-  </si>
-  <si>
-    <t>十号配电室</t>
-  </si>
-  <si>
-    <t>10号变压器</t>
-  </si>
-  <si>
-    <t>USER</t>
-  </si>
-  <si>
-    <t>jldgxcx</t>
-  </si>
-  <si>
-    <t>PASSWORD</t>
-  </si>
-  <si>
-    <t>Jldg123654.</t>
-  </si>
-  <si>
-    <t>HOST</t>
-  </si>
-  <si>
-    <t>xs.jldg.com</t>
-  </si>
-  <si>
-    <t>DATABASE</t>
-  </si>
-  <si>
-    <t>energy</t>
-  </si>
-  <si>
-    <t>192.168.40.19</t>
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
 </sst>
@@ -787,7 +812,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -823,6 +848,12 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1131,7 +1162,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M130"/>
+  <dimension ref="A1:M132"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="11.625" style="3" customWidth="1"/>
@@ -4755,26 +4786,26 @@
       <c r="A89" s="5">
         <v>96</v>
       </c>
-      <c r="B89" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="C89" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="D89" s="8" t="s">
-        <v>141</v>
+      <c r="B89" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="C89" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="D89" s="11" t="s">
+        <v>199</v>
       </c>
       <c r="E89" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F89" s="5" t="s">
-        <v>101</v>
+      <c r="F89" s="11" t="s">
+        <v>201</v>
       </c>
       <c r="G89" s="5">
         <v>502</v>
       </c>
       <c r="H89" s="5">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I89" s="5">
         <v>18</v>
@@ -4796,26 +4827,26 @@
       <c r="A90" s="5">
         <v>97</v>
       </c>
-      <c r="B90" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="C90" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="D90" s="5" t="s">
-        <v>142</v>
+      <c r="B90" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="C90" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="D90" s="11" t="s">
+        <v>200</v>
       </c>
       <c r="E90" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F90" s="5" t="s">
-        <v>134</v>
+      <c r="F90" s="11" t="s">
+        <v>201</v>
       </c>
       <c r="G90" s="5">
         <v>502</v>
       </c>
       <c r="H90" s="5">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="I90" s="5">
         <v>18</v>
@@ -4838,25 +4869,25 @@
         <v>98</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>143</v>
+        <v>98</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>144</v>
+        <v>99</v>
       </c>
       <c r="D91" s="8" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="E91" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F91" s="5" t="s">
-        <v>146</v>
+        <v>101</v>
       </c>
       <c r="G91" s="5">
         <v>502</v>
       </c>
       <c r="H91" s="5">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="I91" s="5">
         <v>18</v>
@@ -4879,25 +4910,25 @@
         <v>99</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>143</v>
+        <v>98</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="D92" s="5" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="E92" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F92" s="5" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="G92" s="5">
         <v>502</v>
       </c>
       <c r="H92" s="5">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="I92" s="5">
         <v>18</v>
@@ -4925,20 +4956,20 @@
       <c r="C93" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="D93" s="5" t="s">
-        <v>148</v>
+      <c r="D93" s="13" t="s">
+        <v>205</v>
       </c>
       <c r="E93" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F93" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G93" s="5">
         <v>502</v>
       </c>
       <c r="H93" s="5">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="I93" s="5">
         <v>18</v>
@@ -4966,20 +4997,20 @@
       <c r="C94" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="D94" s="8" t="s">
-        <v>149</v>
+      <c r="D94" s="5" t="s">
+        <v>146</v>
       </c>
       <c r="E94" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F94" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G94" s="5">
         <v>502</v>
       </c>
       <c r="H94" s="5">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="I94" s="5">
         <v>18</v>
@@ -5007,20 +5038,20 @@
       <c r="C95" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="D95" s="8" t="s">
-        <v>150</v>
+      <c r="D95" s="11" t="s">
+        <v>206</v>
       </c>
       <c r="E95" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F95" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G95" s="5">
         <v>502</v>
       </c>
       <c r="H95" s="5">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="I95" s="5">
         <v>18</v>
@@ -5049,19 +5080,19 @@
         <v>144</v>
       </c>
       <c r="D96" s="8" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E96" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F96" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G96" s="5">
         <v>502</v>
       </c>
       <c r="H96" s="5">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I96" s="5">
         <v>18</v>
@@ -5089,20 +5120,20 @@
       <c r="C97" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="D97" s="5" t="s">
-        <v>152</v>
+      <c r="D97" s="8" t="s">
+        <v>148</v>
       </c>
       <c r="E97" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F97" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G97" s="5">
         <v>502</v>
       </c>
       <c r="H97" s="5">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="I97" s="5">
         <v>18</v>
@@ -5131,19 +5162,19 @@
         <v>144</v>
       </c>
       <c r="D98" s="8" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="E98" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F98" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G98" s="5">
         <v>502</v>
       </c>
       <c r="H98" s="5">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="I98" s="5">
         <v>18</v>
@@ -5172,19 +5203,19 @@
         <v>144</v>
       </c>
       <c r="D99" s="5" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="E99" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F99" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G99" s="5">
         <v>502</v>
       </c>
       <c r="H99" s="5">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I99" s="5">
         <v>18</v>
@@ -5213,19 +5244,19 @@
         <v>144</v>
       </c>
       <c r="D100" s="8" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="E100" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F100" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G100" s="5">
         <v>502</v>
       </c>
       <c r="H100" s="5">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="I100" s="5">
         <v>18</v>
@@ -5253,20 +5284,20 @@
       <c r="C101" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="D101" s="5" t="s">
-        <v>156</v>
+      <c r="D101" s="13" t="s">
+        <v>203</v>
       </c>
       <c r="E101" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F101" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G101" s="5">
         <v>502</v>
       </c>
       <c r="H101" s="5">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="I101" s="5">
         <v>18</v>
@@ -5285,90 +5316,90 @@
       </c>
     </row>
     <row r="102" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A102" s="8">
-        <v>110</v>
+      <c r="A102" s="5">
+        <v>109</v>
       </c>
       <c r="B102" s="5" t="s">
         <v>143</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D102" s="9" t="s">
-        <v>157</v>
+        <v>144</v>
+      </c>
+      <c r="D102" s="13" t="s">
+        <v>204</v>
       </c>
       <c r="E102" s="5" t="s">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="F102" s="5" t="s">
-        <v>158</v>
+        <v>145</v>
       </c>
       <c r="G102" s="5">
-        <v>102</v>
-      </c>
-      <c r="H102" s="5" t="s">
-        <v>51</v>
+        <v>502</v>
+      </c>
+      <c r="H102" s="5">
+        <v>29</v>
       </c>
       <c r="I102" s="5">
-        <v>500</v>
+        <v>18</v>
       </c>
       <c r="J102" s="5">
         <v>4</v>
       </c>
       <c r="K102" s="4" t="s">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="L102" s="4">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="M102" s="4" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="103" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A103" s="8">
-        <v>111</v>
+      <c r="A103" s="5">
+        <v>110</v>
       </c>
       <c r="B103" s="5" t="s">
         <v>143</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D103" s="7" t="s">
-        <v>159</v>
+        <v>144</v>
+      </c>
+      <c r="D103" s="5" t="s">
+        <v>152</v>
       </c>
       <c r="E103" s="5" t="s">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="F103" s="5" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="G103" s="5">
-        <v>102</v>
-      </c>
-      <c r="H103" s="5" t="s">
-        <v>51</v>
+        <v>502</v>
+      </c>
+      <c r="H103" s="5">
+        <v>13</v>
       </c>
       <c r="I103" s="5">
-        <v>500</v>
+        <v>18</v>
       </c>
       <c r="J103" s="5">
         <v>4</v>
       </c>
       <c r="K103" s="4" t="s">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="L103" s="4">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="M103" s="4" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="104" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A104" s="8">
-        <v>112</v>
+      <c r="A104" s="5">
+        <v>111</v>
       </c>
       <c r="B104" s="5" t="s">
         <v>143</v>
@@ -5376,14 +5407,14 @@
       <c r="C104" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D104" s="8" t="s">
-        <v>161</v>
+      <c r="D104" s="9" t="s">
+        <v>153</v>
       </c>
       <c r="E104" s="5" t="s">
         <v>49</v>
       </c>
       <c r="F104" s="5" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="G104" s="5">
         <v>102</v>
@@ -5392,7 +5423,7 @@
         <v>51</v>
       </c>
       <c r="I104" s="5">
-        <v>910</v>
+        <v>500</v>
       </c>
       <c r="J104" s="5">
         <v>4</v>
@@ -5408,90 +5439,90 @@
       </c>
     </row>
     <row r="105" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A105" s="8">
-        <v>113</v>
+      <c r="A105" s="5">
+        <v>112</v>
       </c>
       <c r="B105" s="5" t="s">
         <v>143</v>
       </c>
       <c r="C105" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="D105" s="10" t="s">
-        <v>163</v>
+        <v>47</v>
+      </c>
+      <c r="D105" s="7" t="s">
+        <v>155</v>
       </c>
       <c r="E105" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F105" s="11" t="s">
-        <v>201</v>
+        <v>49</v>
+      </c>
+      <c r="F105" s="5" t="s">
+        <v>156</v>
       </c>
       <c r="G105" s="5">
-        <v>502</v>
-      </c>
-      <c r="H105" s="5">
-        <v>18</v>
+        <v>102</v>
+      </c>
+      <c r="H105" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="I105" s="5">
-        <v>18</v>
+        <v>500</v>
       </c>
       <c r="J105" s="5">
         <v>4</v>
       </c>
       <c r="K105" s="4" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="L105" s="4">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="M105" s="4" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="106" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A106" s="8">
-        <v>114</v>
+      <c r="A106" s="5">
+        <v>113</v>
       </c>
       <c r="B106" s="5" t="s">
         <v>143</v>
       </c>
       <c r="C106" s="5" t="s">
-        <v>144</v>
+        <v>47</v>
       </c>
       <c r="D106" s="8" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="E106" s="5" t="s">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="F106" s="5" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="G106" s="5">
-        <v>502</v>
-      </c>
-      <c r="H106" s="5">
-        <v>40</v>
+        <v>102</v>
+      </c>
+      <c r="H106" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="I106" s="5">
-        <v>18</v>
+        <v>910</v>
       </c>
       <c r="J106" s="5">
         <v>4</v>
       </c>
       <c r="K106" s="4" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="L106" s="4">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="M106" s="4" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="107" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A107" s="8">
-        <v>115</v>
+      <c r="A107" s="5">
+        <v>114</v>
       </c>
       <c r="B107" s="5" t="s">
         <v>143</v>
@@ -5499,20 +5530,20 @@
       <c r="C107" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="D107" s="8" t="s">
-        <v>165</v>
+      <c r="D107" s="10" t="s">
+        <v>159</v>
       </c>
       <c r="E107" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F107" s="5" t="s">
-        <v>146</v>
+      <c r="F107" s="11" t="s">
+        <v>196</v>
       </c>
       <c r="G107" s="5">
         <v>502</v>
       </c>
       <c r="H107" s="5">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="I107" s="5">
         <v>18</v>
@@ -5531,8 +5562,8 @@
       </c>
     </row>
     <row r="108" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A108" s="8">
-        <v>116</v>
+      <c r="A108" s="5">
+        <v>115</v>
       </c>
       <c r="B108" s="5" t="s">
         <v>143</v>
@@ -5540,20 +5571,20 @@
       <c r="C108" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="D108" s="5" t="s">
-        <v>166</v>
+      <c r="D108" s="8" t="s">
+        <v>160</v>
       </c>
       <c r="E108" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F108" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G108" s="5">
         <v>502</v>
       </c>
       <c r="H108" s="5">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="I108" s="5">
         <v>18</v>
@@ -5572,8 +5603,8 @@
       </c>
     </row>
     <row r="109" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A109" s="8">
-        <v>117</v>
+      <c r="A109" s="5">
+        <v>116</v>
       </c>
       <c r="B109" s="5" t="s">
         <v>143</v>
@@ -5582,19 +5613,19 @@
         <v>144</v>
       </c>
       <c r="D109" s="8" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="E109" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F109" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G109" s="5">
         <v>502</v>
       </c>
       <c r="H109" s="5">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="I109" s="5">
         <v>18</v>
@@ -5613,8 +5644,8 @@
       </c>
     </row>
     <row r="110" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A110" s="8">
-        <v>118</v>
+      <c r="A110" s="5">
+        <v>117</v>
       </c>
       <c r="B110" s="5" t="s">
         <v>143</v>
@@ -5622,20 +5653,20 @@
       <c r="C110" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="D110" s="8" t="s">
-        <v>168</v>
+      <c r="D110" s="5" t="s">
+        <v>162</v>
       </c>
       <c r="E110" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F110" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G110" s="5">
         <v>502</v>
       </c>
       <c r="H110" s="5">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="I110" s="5">
         <v>18</v>
@@ -5654,8 +5685,8 @@
       </c>
     </row>
     <row r="111" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A111" s="8">
-        <v>119</v>
+      <c r="A111" s="5">
+        <v>118</v>
       </c>
       <c r="B111" s="5" t="s">
         <v>143</v>
@@ -5663,20 +5694,20 @@
       <c r="C111" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="D111" s="5" t="s">
-        <v>169</v>
+      <c r="D111" s="8" t="s">
+        <v>163</v>
       </c>
       <c r="E111" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F111" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G111" s="5">
         <v>502</v>
       </c>
       <c r="H111" s="5">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="I111" s="5">
         <v>18</v>
@@ -5695,8 +5726,8 @@
       </c>
     </row>
     <row r="112" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A112" s="8">
-        <v>120</v>
+      <c r="A112" s="5">
+        <v>119</v>
       </c>
       <c r="B112" s="5" t="s">
         <v>143</v>
@@ -5704,20 +5735,20 @@
       <c r="C112" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="D112" s="5" t="s">
-        <v>170</v>
+      <c r="D112" s="8" t="s">
+        <v>164</v>
       </c>
       <c r="E112" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F112" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G112" s="5">
         <v>502</v>
       </c>
       <c r="H112" s="5">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="I112" s="5">
         <v>18</v>
@@ -5736,8 +5767,8 @@
       </c>
     </row>
     <row r="113" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A113" s="8">
-        <v>121</v>
+      <c r="A113" s="5">
+        <v>120</v>
       </c>
       <c r="B113" s="5" t="s">
         <v>143</v>
@@ -5746,19 +5777,19 @@
         <v>144</v>
       </c>
       <c r="D113" s="5" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="E113" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F113" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G113" s="5">
         <v>502</v>
       </c>
       <c r="H113" s="5">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I113" s="5">
         <v>18</v>
@@ -5777,49 +5808,49 @@
       </c>
     </row>
     <row r="114" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A114" s="8">
-        <v>123</v>
+      <c r="A114" s="5">
+        <v>121</v>
       </c>
       <c r="B114" s="5" t="s">
         <v>143</v>
       </c>
       <c r="C114" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D114" s="9" t="s">
-        <v>172</v>
+        <v>144</v>
+      </c>
+      <c r="D114" s="5" t="s">
+        <v>166</v>
       </c>
       <c r="E114" s="5" t="s">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="F114" s="5" t="s">
-        <v>173</v>
+        <v>145</v>
       </c>
       <c r="G114" s="5">
-        <v>102</v>
-      </c>
-      <c r="H114" s="5" t="s">
-        <v>51</v>
+        <v>502</v>
+      </c>
+      <c r="H114" s="5">
+        <v>5</v>
       </c>
       <c r="I114" s="5">
-        <v>500</v>
+        <v>18</v>
       </c>
       <c r="J114" s="5">
         <v>4</v>
       </c>
       <c r="K114" s="4" t="s">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="L114" s="4">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="M114" s="4" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="115" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A115" s="8">
-        <v>124</v>
+      <c r="A115" s="5">
+        <v>122</v>
       </c>
       <c r="B115" s="5" t="s">
         <v>143</v>
@@ -5827,20 +5858,20 @@
       <c r="C115" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="D115" s="8" t="s">
-        <v>174</v>
+      <c r="D115" s="5" t="s">
+        <v>167</v>
       </c>
       <c r="E115" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F115" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G115" s="5">
         <v>502</v>
       </c>
       <c r="H115" s="5">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="I115" s="5">
         <v>18</v>
@@ -5859,49 +5890,49 @@
       </c>
     </row>
     <row r="116" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A116" s="8">
-        <v>125</v>
+      <c r="A116" s="5">
+        <v>123</v>
       </c>
       <c r="B116" s="5" t="s">
         <v>143</v>
       </c>
       <c r="C116" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="D116" s="8" t="s">
-        <v>175</v>
+        <v>47</v>
+      </c>
+      <c r="D116" s="9" t="s">
+        <v>168</v>
       </c>
       <c r="E116" s="5" t="s">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="F116" s="5" t="s">
-        <v>146</v>
+        <v>169</v>
       </c>
       <c r="G116" s="5">
-        <v>502</v>
-      </c>
-      <c r="H116" s="5">
-        <v>41</v>
+        <v>102</v>
+      </c>
+      <c r="H116" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="I116" s="5">
-        <v>18</v>
+        <v>500</v>
       </c>
       <c r="J116" s="5">
         <v>4</v>
       </c>
       <c r="K116" s="4" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="L116" s="4">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="M116" s="4" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="117" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A117" s="8">
-        <v>126</v>
+      <c r="A117" s="5">
+        <v>124</v>
       </c>
       <c r="B117" s="5" t="s">
         <v>143</v>
@@ -5910,19 +5941,19 @@
         <v>144</v>
       </c>
       <c r="D117" s="8" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="E117" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F117" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G117" s="5">
         <v>502</v>
       </c>
       <c r="H117" s="5">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="I117" s="5">
         <v>18</v>
@@ -5941,8 +5972,8 @@
       </c>
     </row>
     <row r="118" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A118" s="8">
-        <v>127</v>
+      <c r="A118" s="5">
+        <v>125</v>
       </c>
       <c r="B118" s="5" t="s">
         <v>143</v>
@@ -5950,20 +5981,20 @@
       <c r="C118" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="D118" s="5" t="s">
-        <v>177</v>
+      <c r="D118" s="8" t="s">
+        <v>171</v>
       </c>
       <c r="E118" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F118" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G118" s="5">
         <v>502</v>
       </c>
       <c r="H118" s="5">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="I118" s="5">
         <v>18</v>
@@ -5982,41 +6013,41 @@
       </c>
     </row>
     <row r="119" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A119" s="8">
-        <v>130</v>
+      <c r="A119" s="5">
+        <v>126</v>
       </c>
       <c r="B119" s="5" t="s">
-        <v>178</v>
+        <v>143</v>
       </c>
       <c r="C119" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D119" s="9" t="s">
-        <v>179</v>
+        <v>144</v>
+      </c>
+      <c r="D119" s="8" t="s">
+        <v>172</v>
       </c>
       <c r="E119" s="5" t="s">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="F119" s="5" t="s">
-        <v>180</v>
+        <v>145</v>
       </c>
       <c r="G119" s="5">
-        <v>102</v>
-      </c>
-      <c r="H119" s="5" t="s">
-        <v>51</v>
+        <v>502</v>
+      </c>
+      <c r="H119" s="5">
+        <v>42</v>
       </c>
       <c r="I119" s="5">
-        <v>500</v>
+        <v>18</v>
       </c>
       <c r="J119" s="5">
         <v>4</v>
       </c>
       <c r="K119" s="4" t="s">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="L119" s="4">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="M119" s="4" t="s">
         <v>19</v>
@@ -6024,7 +6055,7 @@
     </row>
     <row r="120" spans="1:13" x14ac:dyDescent="0.15">
       <c r="A120" s="5">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B120" s="5" t="s">
         <v>143</v>
@@ -6033,136 +6064,136 @@
         <v>144</v>
       </c>
       <c r="D120" s="5" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="E120" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F120" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G120" s="5">
         <v>502</v>
       </c>
       <c r="H120" s="5">
+        <v>19</v>
+      </c>
+      <c r="I120" s="5">
+        <v>18</v>
+      </c>
+      <c r="J120" s="5">
+        <v>4</v>
+      </c>
+      <c r="K120" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="L120" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="M120" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="121" spans="1:13" x14ac:dyDescent="0.15">
+      <c r="A121" s="5">
+        <v>128</v>
+      </c>
+      <c r="B121" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="C121" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D121" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="E121" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F121" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="G121" s="5">
+        <v>102</v>
+      </c>
+      <c r="H121" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="I121" s="5">
+        <v>500</v>
+      </c>
+      <c r="J121" s="5">
+        <v>4</v>
+      </c>
+      <c r="K121" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="L121" s="4">
+        <v>1</v>
+      </c>
+      <c r="M121" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="122" spans="1:13" x14ac:dyDescent="0.15">
+      <c r="A122" s="5">
+        <v>129</v>
+      </c>
+      <c r="B122" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="C122" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="D122" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="E122" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F122" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="G122" s="5">
+        <v>502</v>
+      </c>
+      <c r="H122" s="5">
         <v>27</v>
       </c>
-      <c r="I120" s="5">
-        <v>18</v>
-      </c>
-      <c r="J120" s="5">
-        <v>4</v>
-      </c>
-      <c r="K120" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="L120" s="4">
-        <v>0.1</v>
-      </c>
-      <c r="M120" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="121" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A121" s="10">
-        <v>143</v>
-      </c>
-      <c r="B121" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C121" s="5" t="s">
+      <c r="I122" s="5">
+        <v>18</v>
+      </c>
+      <c r="J122" s="5">
+        <v>4</v>
+      </c>
+      <c r="K122" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="L122" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="M122" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="123" spans="1:13" x14ac:dyDescent="0.15">
+      <c r="A123" s="5">
+        <v>130</v>
+      </c>
+      <c r="B123" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C123" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D121" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="E121" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F121" s="5" t="s">
+      <c r="D123" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="E123" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F123" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="G121" s="5">
-        <v>502</v>
-      </c>
-      <c r="H121" s="5">
-        <v>100</v>
-      </c>
-      <c r="I121" s="5">
-        <v>18</v>
-      </c>
-      <c r="J121" s="5">
-        <v>4</v>
-      </c>
-      <c r="K121" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="L121" s="4">
-        <v>0.1</v>
-      </c>
-      <c r="M121" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="122" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A122" s="10">
-        <v>144</v>
-      </c>
-      <c r="B122" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C122" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D122" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="E122" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F122" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G122" s="5">
-        <v>502</v>
-      </c>
-      <c r="H122" s="5">
-        <v>100</v>
-      </c>
-      <c r="I122" s="5">
-        <v>18</v>
-      </c>
-      <c r="J122" s="5">
-        <v>4</v>
-      </c>
-      <c r="K122" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="L122" s="4">
-        <v>0.1</v>
-      </c>
-      <c r="M122" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="123" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A123" s="10">
-        <v>145</v>
-      </c>
-      <c r="B123" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C123" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D123" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="E123" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F123" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="G123" s="5">
         <v>502</v>
@@ -6187,23 +6218,23 @@
       </c>
     </row>
     <row r="124" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A124" s="10">
-        <v>146</v>
+      <c r="A124" s="5">
+        <v>131</v>
       </c>
       <c r="B124" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C124" s="5" t="s">
-        <v>76</v>
+        <v>27</v>
       </c>
       <c r="D124" s="5" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="E124" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F124" s="5" t="s">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="G124" s="5">
         <v>502</v>
@@ -6228,23 +6259,23 @@
       </c>
     </row>
     <row r="125" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A125" s="10">
-        <v>147</v>
+      <c r="A125" s="5">
+        <v>132</v>
       </c>
       <c r="B125" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C125" s="5" t="s">
-        <v>62</v>
+        <v>14</v>
       </c>
       <c r="D125" s="5" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="E125" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F125" s="5" t="s">
-        <v>64</v>
+        <v>17</v>
       </c>
       <c r="G125" s="5">
         <v>502</v>
@@ -6269,23 +6300,23 @@
       </c>
     </row>
     <row r="126" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A126" s="10">
-        <v>148</v>
+      <c r="A126" s="5">
+        <v>133</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>98</v>
+        <v>13</v>
       </c>
       <c r="C126" s="5" t="s">
-        <v>99</v>
+        <v>76</v>
       </c>
       <c r="D126" s="5" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="E126" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F126" s="5" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="G126" s="5">
         <v>502</v>
@@ -6310,23 +6341,23 @@
       </c>
     </row>
     <row r="127" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A127" s="10">
-        <v>149</v>
+      <c r="A127" s="5">
+        <v>134</v>
       </c>
       <c r="B127" s="5" t="s">
-        <v>98</v>
+        <v>13</v>
       </c>
       <c r="C127" s="5" t="s">
-        <v>103</v>
+        <v>62</v>
       </c>
       <c r="D127" s="5" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="E127" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F127" s="5" t="s">
-        <v>105</v>
+        <v>64</v>
       </c>
       <c r="G127" s="5">
         <v>502</v>
@@ -6351,23 +6382,23 @@
       </c>
     </row>
     <row r="128" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A128" s="10">
-        <v>150</v>
+      <c r="A128" s="5">
+        <v>135</v>
       </c>
       <c r="B128" s="5" t="s">
         <v>98</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>132</v>
+        <v>99</v>
       </c>
       <c r="D128" s="5" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="E128" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F128" s="5" t="s">
-        <v>134</v>
+        <v>101</v>
       </c>
       <c r="G128" s="5">
         <v>502</v>
@@ -6392,23 +6423,23 @@
       </c>
     </row>
     <row r="129" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A129" s="10">
-        <v>151</v>
+      <c r="A129" s="5">
+        <v>136</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>143</v>
+        <v>98</v>
       </c>
       <c r="C129" s="5" t="s">
-        <v>144</v>
+        <v>103</v>
       </c>
       <c r="D129" s="5" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E129" s="5" t="s">
         <v>16</v>
       </c>
       <c r="F129" s="5" t="s">
-        <v>146</v>
+        <v>105</v>
       </c>
       <c r="G129" s="5">
         <v>502</v>
@@ -6433,49 +6464,131 @@
       </c>
     </row>
     <row r="130" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A130" s="10">
-        <v>152</v>
+      <c r="A130" s="5">
+        <v>137</v>
       </c>
       <c r="B130" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C130" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="D130" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="E130" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F130" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="G130" s="5">
+        <v>502</v>
+      </c>
+      <c r="H130" s="5">
+        <v>100</v>
+      </c>
+      <c r="I130" s="5">
+        <v>18</v>
+      </c>
+      <c r="J130" s="5">
+        <v>4</v>
+      </c>
+      <c r="K130" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="L130" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="M130" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="131" spans="1:13" x14ac:dyDescent="0.15">
+      <c r="A131" s="5">
+        <v>138</v>
+      </c>
+      <c r="B131" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="C130" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="D130" s="5" t="s">
-        <v>192</v>
-      </c>
-      <c r="E130" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F130" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="G130" s="5">
-        <v>502</v>
-      </c>
-      <c r="H130" s="5">
+      <c r="C131" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="D131" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="E131" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F131" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="G131" s="5">
+        <v>502</v>
+      </c>
+      <c r="H131" s="5">
+        <v>100</v>
+      </c>
+      <c r="I131" s="5">
+        <v>18</v>
+      </c>
+      <c r="J131" s="5">
+        <v>4</v>
+      </c>
+      <c r="K131" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="L131" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="M131" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="132" spans="1:13" x14ac:dyDescent="0.15">
+      <c r="A132" s="5">
+        <v>139</v>
+      </c>
+      <c r="B132" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="C132" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="D132" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="E132" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F132" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="G132" s="5">
+        <v>502</v>
+      </c>
+      <c r="H132" s="5">
         <v>101</v>
       </c>
-      <c r="I130" s="5">
-        <v>18</v>
-      </c>
-      <c r="J130" s="5">
-        <v>4</v>
-      </c>
-      <c r="K130" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="L130" s="4">
-        <v>0.1</v>
-      </c>
-      <c r="M130" s="4" t="s">
+      <c r="I132" s="5">
+        <v>18</v>
+      </c>
+      <c r="J132" s="5">
+        <v>4</v>
+      </c>
+      <c r="K132" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="L132" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="M132" s="4" t="s">
         <v>19</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J129">
-    <sortCondition ref="A2:A129"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J131">
+    <sortCondition ref="A2:A131"/>
   </sortState>
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6494,26 +6607,26 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A3" s="1" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.15">
@@ -6526,10 +6639,10 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A5" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>200</v>
+        <v>195</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>